<commit_message>
feat: generalize construction VFX and stabilize navigation
Apply contour-based construction effects and vehicle lasers through the shared building lifecycle, with owned Niagara assets and shape caches. Include current Mass navigation and teleport ground validation fixes, authoring tools, and project records. Make construction tools recreate their output directories after cleanup.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeVfx.xlsx
+++ b/data/Excel/GuLiStrikeVfx.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
     <t>id</t>
   </si>
@@ -437,6 +437,51 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/Buildings/Construction/M_BuildingPlacementGrid.M_BuildingPlacementGrid</t>
+  </si>
+  <si>
+    <t>BuildingConstructionComplete</t>
+  </si>
+  <si>
+    <t>矿厂完工底部UpgradeGlow一次性完整闪光</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Buildings/Construction/NS_ConstructionComplete.NS_ConstructionComplete</t>
+  </si>
+  <si>
+    <t>BuildingConstructionTopLoop</t>
+  </si>
+  <si>
+    <t>矿厂屋檐淡青绿呼吸光柱、漂浮粒子与独立电火花</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Buildings/Construction/NS_ConstructionTopLoop.NS_ConstructionTopLoop</t>
+  </si>
+  <si>
+    <t>BuildingConstructionLaser</t>
+  </si>
+  <si>
+    <t>建造车左右紫色激光、蓝白落点火花</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Buildings/Construction/NS_ConstructionLaser_Purple.NS_ConstructionLaser_Purple</t>
+  </si>
+  <si>
+    <t>BuildingConstructionColumnTail</t>
+  </si>
+  <si>
+    <t>施工弱光柱材质，提取UpgradeGlow残尾</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Buildings/Construction/M_ConstructionColumnTail.M_ConstructionColumnTail</t>
+  </si>
+  <si>
+    <t>BuildingConstructionMote</t>
+  </si>
+  <si>
+    <t>施工向上漂浮三角粒子材质</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Buildings/Construction/M_ConstructionMote.M_ConstructionMote</t>
   </si>
 </sst>
 </file>
@@ -1808,6 +1853,121 @@
         <v>1</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46">
+        <v>43</v>
+      </c>
+      <c r="B46" t="s">
+        <v>141</v>
+      </c>
+      <c r="C46" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" t="s">
+        <v>143</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>44</v>
+      </c>
+      <c r="B47" t="s">
+        <v>144</v>
+      </c>
+      <c r="C47" t="s">
+        <v>145</v>
+      </c>
+      <c r="D47" t="s">
+        <v>146</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>45</v>
+      </c>
+      <c r="B48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C48" t="s">
+        <v>148</v>
+      </c>
+      <c r="D48" t="s">
+        <v>149</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>46</v>
+      </c>
+      <c r="B49" t="s">
+        <v>150</v>
+      </c>
+      <c r="C49" t="s">
+        <v>151</v>
+      </c>
+      <c r="D49" t="s">
+        <v>152</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>47</v>
+      </c>
+      <c r="B50" t="s">
+        <v>153</v>
+      </c>
+      <c r="C50" t="s">
+        <v>154</v>
+      </c>
+      <c r="D50" t="s">
+        <v>155</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>